<commit_message>
Complete repository for statistical analysis
</commit_message>
<xml_diff>
--- a/Branchlet/experiment note.xlsx
+++ b/Branchlet/experiment note.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10125"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud-my.sharepoint.com/personal/haninhn_student_unimelb_edu_au/Documents/Documents/Chapter 2/Chapter 2 data/Branchlet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{75BA6992-2943-534C-A194-6274ADBAC4E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34FD8D9C-5A6E-4147-8703-7EDF76D383BC}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{75BA6992-2943-534C-A194-6274ADBAC4E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D5DF9DC-24D4-E14D-8CF7-615D18A29C85}"/>
   <bookViews>
-    <workbookView xWindow="864" yWindow="-108" windowWidth="22284" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5920" yWindow="-18900" windowWidth="22280" windowHeight="14620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -192,9 +192,6 @@
     <t>Source.Name</t>
   </si>
   <si>
-    <t>0422_01</t>
-  </si>
-  <si>
     <t>2 first thermal videos</t>
   </si>
   <si>
@@ -273,9 +270,6 @@
     <t>No visual footage</t>
   </si>
   <si>
-    <t>0506_01</t>
-  </si>
-  <si>
     <t>0506_03</t>
   </si>
   <si>
@@ -496,6 +490,12 @@
   </si>
   <si>
     <t>100 kW C2</t>
+  </si>
+  <si>
+    <t>0421_01</t>
+  </si>
+  <si>
+    <t>0505_01</t>
   </si>
 </sst>
 </file>
@@ -679,13 +679,30 @@
     <xf numFmtId="20" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="20" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="16" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -700,20 +717,18 @@
     <xf numFmtId="16" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="20" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -723,27 +738,12 @@
     <xf numFmtId="16" fontId="0" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="0" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="16" fontId="0" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1025,35 +1025,35 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M79"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.33203125" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="9" customWidth="1"/>
     <col min="5" max="5" width="6.6640625" customWidth="1"/>
-    <col min="6" max="6" width="6.109375" customWidth="1"/>
-    <col min="7" max="7" width="6.77734375" customWidth="1"/>
+    <col min="6" max="6" width="6.1640625" customWidth="1"/>
+    <col min="7" max="7" width="6.83203125" customWidth="1"/>
     <col min="8" max="8" width="13.6640625" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="10" width="15.44140625" customWidth="1"/>
+    <col min="10" max="10" width="15.5" customWidth="1"/>
     <col min="11" max="11" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="C1" s="1"/>
       <c r="D1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="13" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D2" s="13" t="s">
         <v>1</v>
@@ -1080,11 +1080,11 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" s="17" t="s">
-        <v>146</v>
-      </c>
-      <c r="B3" s="18">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3" s="26" t="s">
+        <v>144</v>
+      </c>
+      <c r="B3" s="27">
         <v>45743</v>
       </c>
       <c r="C3" s="2">
@@ -1122,9 +1122,9 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4" s="17"/>
-      <c r="B4" s="18"/>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" s="26"/>
+      <c r="B4" s="27"/>
       <c r="C4" s="4">
         <v>2</v>
       </c>
@@ -1152,9 +1152,9 @@
       </c>
       <c r="K4" s="4"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A5" s="17"/>
-      <c r="B5" s="18"/>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5" s="26"/>
+      <c r="B5" s="27"/>
       <c r="C5" s="2">
         <v>3</v>
       </c>
@@ -1182,9 +1182,9 @@
       </c>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" s="17"/>
-      <c r="B6" s="18"/>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A6" s="26"/>
+      <c r="B6" s="27"/>
       <c r="C6" s="4">
         <v>4</v>
       </c>
@@ -1212,9 +1212,9 @@
       </c>
       <c r="K6" s="4"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" s="17"/>
-      <c r="B7" s="18"/>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A7" s="26"/>
+      <c r="B7" s="27"/>
       <c r="C7" s="2">
         <v>5</v>
       </c>
@@ -1242,9 +1242,9 @@
       </c>
       <c r="K7" s="2"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A8" s="17"/>
-      <c r="B8" s="18"/>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A8" s="26"/>
+      <c r="B8" s="27"/>
       <c r="C8" s="4">
         <v>6</v>
       </c>
@@ -1265,16 +1265,16 @@
         <v>19</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="J8" s="4">
         <v>6</v>
       </c>
       <c r="K8" s="4"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A9" s="17"/>
-      <c r="B9" s="18"/>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A9" s="26"/>
+      <c r="B9" s="27"/>
       <c r="C9" s="2">
         <v>7</v>
       </c>
@@ -1302,9 +1302,9 @@
       </c>
       <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A10" s="17"/>
-      <c r="B10" s="18"/>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A10" s="26"/>
+      <c r="B10" s="27"/>
       <c r="C10" s="4">
         <v>8</v>
       </c>
@@ -1332,9 +1332,9 @@
       </c>
       <c r="K10" s="4"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" s="17"/>
-      <c r="B11" s="18">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A11" s="26"/>
+      <c r="B11" s="27">
         <v>45748</v>
       </c>
       <c r="C11" s="2">
@@ -1364,9 +1364,9 @@
       </c>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="17"/>
-      <c r="B12" s="18"/>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A12" s="26"/>
+      <c r="B12" s="27"/>
       <c r="C12" s="4">
         <v>10</v>
       </c>
@@ -1394,9 +1394,9 @@
       </c>
       <c r="K12" s="4"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A13" s="17"/>
-      <c r="B13" s="18"/>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A13" s="26"/>
+      <c r="B13" s="27"/>
       <c r="C13" s="2">
         <v>11</v>
       </c>
@@ -1424,9 +1424,9 @@
       </c>
       <c r="K13" s="2"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A14" s="17"/>
-      <c r="B14" s="18"/>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A14" s="26"/>
+      <c r="B14" s="27"/>
       <c r="C14" s="4">
         <v>12</v>
       </c>
@@ -1454,9 +1454,9 @@
       </c>
       <c r="K14" s="4"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" s="17"/>
-      <c r="B15" s="18"/>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A15" s="26"/>
+      <c r="B15" s="27"/>
       <c r="C15" s="2">
         <v>13</v>
       </c>
@@ -1484,9 +1484,9 @@
       </c>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A16" s="17"/>
-      <c r="B16" s="18"/>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A16" s="26"/>
+      <c r="B16" s="27"/>
       <c r="C16" s="4">
         <v>14</v>
       </c>
@@ -1514,9 +1514,9 @@
       </c>
       <c r="K16" s="4"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A17" s="17"/>
-      <c r="B17" s="18"/>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A17" s="26"/>
+      <c r="B17" s="27"/>
       <c r="C17" s="2">
         <v>15</v>
       </c>
@@ -1544,9 +1544,9 @@
       </c>
       <c r="K17" s="2"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A18" s="17"/>
-      <c r="B18" s="18"/>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A18" s="26"/>
+      <c r="B18" s="27"/>
       <c r="C18" s="4">
         <v>16</v>
       </c>
@@ -1574,9 +1574,9 @@
       </c>
       <c r="K18" s="4"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A19" s="17"/>
-      <c r="B19" s="18"/>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A19" s="26"/>
+      <c r="B19" s="27"/>
       <c r="C19" s="2">
         <v>17</v>
       </c>
@@ -1604,9 +1604,9 @@
       </c>
       <c r="K19" s="2"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A20" s="17"/>
-      <c r="B20" s="18"/>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A20" s="26"/>
+      <c r="B20" s="27"/>
       <c r="C20" s="4">
         <v>18</v>
       </c>
@@ -1634,9 +1634,9 @@
       </c>
       <c r="K20" s="4"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A21" s="17"/>
-      <c r="B21" s="18"/>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A21" s="26"/>
+      <c r="B21" s="27"/>
       <c r="C21" s="2">
         <v>19</v>
       </c>
@@ -1666,9 +1666,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A22" s="17"/>
-      <c r="B22" s="18"/>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A22" s="26"/>
+      <c r="B22" s="27"/>
       <c r="C22" s="4">
         <v>20</v>
       </c>
@@ -1696,11 +1696,11 @@
       </c>
       <c r="K22" s="4"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A23" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="B23" s="19">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A23" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" s="28">
         <v>45763</v>
       </c>
       <c r="C23" s="7">
@@ -1720,25 +1720,25 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>51</v>
+        <v>151</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J23" s="7">
         <v>6</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L23">
         <f>SUM(J23:J32)</f>
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A24" s="17"/>
-      <c r="B24" s="19"/>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A24" s="26"/>
+      <c r="B24" s="28"/>
       <c r="C24" s="7">
         <v>22</v>
       </c>
@@ -1756,19 +1756,19 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J24" s="7">
         <v>9</v>
       </c>
       <c r="K24" s="7"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A25" s="17"/>
-      <c r="B25" s="19"/>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A25" s="26"/>
+      <c r="B25" s="28"/>
       <c r="C25" s="7">
         <v>23</v>
       </c>
@@ -1786,19 +1786,19 @@
         <v>7.6388888888888618E-3</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J25" s="7">
         <v>5</v>
       </c>
       <c r="K25" s="7"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A26" s="17"/>
-      <c r="B26" s="19"/>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A26" s="26"/>
+      <c r="B26" s="28"/>
       <c r="C26" s="7">
         <v>24</v>
       </c>
@@ -1816,19 +1816,19 @@
         <v>1.0416666666666741E-2</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J26" s="7">
         <v>3</v>
       </c>
       <c r="K26" s="7"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A27" s="17"/>
-      <c r="B27" s="19"/>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A27" s="26"/>
+      <c r="B27" s="28"/>
       <c r="C27" s="7">
         <v>25</v>
       </c>
@@ -1846,19 +1846,19 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J27" s="7">
         <v>3</v>
       </c>
       <c r="K27" s="7"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A28" s="17"/>
-      <c r="B28" s="19"/>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A28" s="26"/>
+      <c r="B28" s="28"/>
       <c r="C28" s="7">
         <v>26</v>
       </c>
@@ -1876,19 +1876,19 @@
         <v>1.0416666666666741E-2</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J28" s="7">
         <v>5</v>
       </c>
       <c r="K28" s="7"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A29" s="17"/>
-      <c r="B29" s="19"/>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A29" s="26"/>
+      <c r="B29" s="28"/>
       <c r="C29" s="7">
         <v>27</v>
       </c>
@@ -1906,19 +1906,19 @@
         <v>8.3333333333333037E-3</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J29" s="7">
         <v>3</v>
       </c>
       <c r="K29" s="7"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A30" s="17"/>
-      <c r="B30" s="19"/>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A30" s="26"/>
+      <c r="B30" s="28"/>
       <c r="C30" s="7">
         <v>28</v>
       </c>
@@ -1936,19 +1936,19 @@
         <v>6.9444444444444198E-3</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J30" s="7">
         <v>5</v>
       </c>
       <c r="K30" s="7"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A31" s="17"/>
-      <c r="B31" s="19"/>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A31" s="26"/>
+      <c r="B31" s="28"/>
       <c r="C31" s="7">
         <v>29</v>
       </c>
@@ -1966,19 +1966,19 @@
         <v>9.0277777777777457E-3</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J31" s="7">
         <v>4</v>
       </c>
       <c r="K31" s="7"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A32" s="17"/>
-      <c r="B32" s="19"/>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A32" s="26"/>
+      <c r="B32" s="28"/>
       <c r="C32" s="7">
         <v>30</v>
       </c>
@@ -1996,21 +1996,21 @@
         <v>9.7222222222222987E-3</v>
       </c>
       <c r="H32" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J32" s="7">
         <v>6</v>
       </c>
       <c r="K32" s="7"/>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A33" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="B33" s="20">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A33" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="B33" s="29">
         <v>45778</v>
       </c>
       <c r="C33" s="9">
@@ -2030,10 +2030,10 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>78</v>
+        <v>152</v>
       </c>
       <c r="I33" s="9" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J33" s="9">
         <v>2</v>
@@ -2044,9 +2044,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A34" s="17"/>
-      <c r="B34" s="20"/>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A34" s="26"/>
+      <c r="B34" s="29"/>
       <c r="C34" s="9">
         <v>32</v>
       </c>
@@ -2064,19 +2064,19 @@
         <v>1.0416666666666741E-2</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I34" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="J34" s="9">
         <v>4</v>
       </c>
       <c r="K34" s="9"/>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A35" s="17"/>
-      <c r="B35" s="20"/>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A35" s="26"/>
+      <c r="B35" s="29"/>
       <c r="C35" s="9">
         <v>33</v>
       </c>
@@ -2094,21 +2094,21 @@
         <v>1.0416666666666741E-2</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I35" s="9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J35" s="9">
         <v>3</v>
       </c>
       <c r="K35" s="9" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A36" s="17"/>
-      <c r="B36" s="20"/>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A36" s="26"/>
+      <c r="B36" s="29"/>
       <c r="C36" s="9">
         <v>34</v>
       </c>
@@ -2126,19 +2126,19 @@
         <v>1.0416666666666741E-2</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I36" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="J36" s="9">
         <v>3</v>
       </c>
       <c r="K36" s="9"/>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A37" s="17"/>
-      <c r="B37" s="20"/>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A37" s="26"/>
+      <c r="B37" s="29"/>
       <c r="C37" s="9">
         <v>35</v>
       </c>
@@ -2156,19 +2156,19 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H37" s="9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="I37" s="9" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="J37" s="9">
         <v>3</v>
       </c>
       <c r="K37" s="9"/>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A38" s="17"/>
-      <c r="B38" s="20">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A38" s="26"/>
+      <c r="B38" s="29">
         <v>45779</v>
       </c>
       <c r="C38" s="9">
@@ -2188,21 +2188,21 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I38" s="9" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="J38" s="9">
         <v>2</v>
       </c>
       <c r="K38" s="9" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A39" s="17"/>
-      <c r="B39" s="20"/>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A39" s="26"/>
+      <c r="B39" s="29"/>
       <c r="C39" s="9">
         <v>37</v>
       </c>
@@ -2220,19 +2220,19 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="I39" s="9" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J39" s="9">
         <v>3</v>
       </c>
       <c r="K39" s="9"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A40" s="17"/>
-      <c r="B40" s="20"/>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A40" s="26"/>
+      <c r="B40" s="29"/>
       <c r="C40" s="9">
         <v>38</v>
       </c>
@@ -2250,19 +2250,19 @@
         <v>1.0416666666666741E-2</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I40" s="9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J40" s="9">
         <v>2</v>
       </c>
       <c r="K40" s="9"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A41" s="17"/>
-      <c r="B41" s="20"/>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A41" s="26"/>
+      <c r="B41" s="29"/>
       <c r="C41" s="9">
         <v>39</v>
       </c>
@@ -2280,19 +2280,19 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H41" s="9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="I41" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="J41" s="9">
         <v>3</v>
       </c>
       <c r="K41" s="9"/>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A42" s="17"/>
-      <c r="B42" s="20"/>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A42" s="26"/>
+      <c r="B42" s="29"/>
       <c r="C42" s="9">
         <v>40</v>
       </c>
@@ -2310,23 +2310,23 @@
         <v>8.3333333333333037E-3</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I42" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J42" s="9">
         <v>3</v>
       </c>
       <c r="K42" s="9" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A43" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="B43" s="14">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A43" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="B43" s="30">
         <v>45792</v>
       </c>
       <c r="C43" s="10">
@@ -2346,10 +2346,10 @@
         <v>9.0277777777777457E-3</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I43" s="10" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J43" s="10">
         <v>2</v>
@@ -2360,9 +2360,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A44" s="17"/>
-      <c r="B44" s="15"/>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A44" s="26"/>
+      <c r="B44" s="31"/>
       <c r="C44" s="10">
         <v>42</v>
       </c>
@@ -2380,19 +2380,19 @@
         <v>1.0416666666666741E-2</v>
       </c>
       <c r="H44" s="10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J44" s="10">
         <v>2</v>
       </c>
       <c r="K44" s="10"/>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A45" s="17"/>
-      <c r="B45" s="15"/>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A45" s="26"/>
+      <c r="B45" s="31"/>
       <c r="C45" s="10">
         <v>43</v>
       </c>
@@ -2410,19 +2410,19 @@
         <v>8.3333333333333037E-3</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I45" s="10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="J45" s="10">
         <v>3</v>
       </c>
       <c r="K45" s="10"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A46" s="17"/>
-      <c r="B46" s="15"/>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A46" s="26"/>
+      <c r="B46" s="31"/>
       <c r="C46" s="10">
         <v>44</v>
       </c>
@@ -2440,19 +2440,19 @@
         <v>9.0277777777777457E-3</v>
       </c>
       <c r="H46" s="10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="J46" s="10">
         <v>2</v>
       </c>
       <c r="K46" s="10"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A47" s="17"/>
-      <c r="B47" s="14">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A47" s="26"/>
+      <c r="B47" s="30">
         <v>45793</v>
       </c>
       <c r="C47" s="10">
@@ -2472,19 +2472,19 @@
         <v>7.6388888888888618E-3</v>
       </c>
       <c r="H47" s="10" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I47" s="10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="J47" s="10">
         <v>2</v>
       </c>
       <c r="K47" s="10"/>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A48" s="17"/>
-      <c r="B48" s="14"/>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A48" s="26"/>
+      <c r="B48" s="30"/>
       <c r="C48" s="10">
         <v>46</v>
       </c>
@@ -2502,19 +2502,19 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H48" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J48" s="10">
         <v>2</v>
       </c>
       <c r="K48" s="10"/>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A49" s="17"/>
-      <c r="B49" s="14"/>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A49" s="26"/>
+      <c r="B49" s="30"/>
       <c r="C49" s="10">
         <v>47</v>
       </c>
@@ -2532,19 +2532,19 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="I49" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J49" s="10">
         <v>3</v>
       </c>
       <c r="K49" s="10"/>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A50" s="17"/>
-      <c r="B50" s="14"/>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A50" s="26"/>
+      <c r="B50" s="30"/>
       <c r="C50" s="10">
         <v>48</v>
       </c>
@@ -2562,19 +2562,19 @@
         <v>9.7222222222222987E-3</v>
       </c>
       <c r="H50" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="I50" s="10" t="s">
         <v>115</v>
-      </c>
-      <c r="I50" s="10" t="s">
-        <v>117</v>
       </c>
       <c r="J50" s="10">
         <v>2</v>
       </c>
       <c r="K50" s="10"/>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A51" s="17"/>
-      <c r="B51" s="14"/>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A51" s="26"/>
+      <c r="B51" s="30"/>
       <c r="C51" s="10">
         <v>49</v>
       </c>
@@ -2592,19 +2592,19 @@
         <v>6.9444444444444198E-3</v>
       </c>
       <c r="H51" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I51" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="J51" s="10">
         <v>4</v>
       </c>
       <c r="K51" s="10"/>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A52" s="17"/>
-      <c r="B52" s="14"/>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A52" s="26"/>
+      <c r="B52" s="30"/>
       <c r="C52" s="10">
         <v>50</v>
       </c>
@@ -2622,21 +2622,21 @@
         <v>7.6388888888889728E-3</v>
       </c>
       <c r="H52" s="10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="J52" s="10">
         <v>3</v>
       </c>
       <c r="K52" s="10"/>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A53" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="B53" s="16">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A53" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="B53" s="32">
         <v>45794</v>
       </c>
       <c r="C53" s="2">
@@ -2656,10 +2656,10 @@
         <v>9.2361111111111116E-2</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J53" s="2">
         <v>2</v>
@@ -2670,9 +2670,9 @@
         <v>23</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A54" s="17"/>
-      <c r="B54" s="16"/>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A54" s="26"/>
+      <c r="B54" s="32"/>
       <c r="C54" s="2">
         <v>52</v>
       </c>
@@ -2690,19 +2690,19 @@
         <v>1.0416666666666741E-2</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J54" s="2">
         <v>2</v>
       </c>
       <c r="K54" s="2"/>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A55" s="17"/>
-      <c r="B55" s="16"/>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A55" s="26"/>
+      <c r="B55" s="32"/>
       <c r="C55" s="2">
         <v>53</v>
       </c>
@@ -2720,19 +2720,19 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J55" s="2">
         <v>2</v>
       </c>
       <c r="K55" s="2"/>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A56" s="17"/>
-      <c r="B56" s="16"/>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A56" s="26"/>
+      <c r="B56" s="32"/>
       <c r="C56" s="2">
         <v>54</v>
       </c>
@@ -2750,19 +2750,19 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="J56" s="2">
         <v>2</v>
       </c>
       <c r="K56" s="2"/>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A57" s="17"/>
-      <c r="B57" s="16"/>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A57" s="26"/>
+      <c r="B57" s="32"/>
       <c r="C57" s="2">
         <v>55</v>
       </c>
@@ -2780,19 +2780,19 @@
         <v>9.0277777777778567E-3</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="J57" s="2">
         <v>3</v>
       </c>
       <c r="K57" s="2"/>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A58" s="17"/>
-      <c r="B58" s="16"/>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A58" s="26"/>
+      <c r="B58" s="32"/>
       <c r="C58" s="2">
         <v>56</v>
       </c>
@@ -2810,19 +2810,19 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J58" s="2">
         <v>2</v>
       </c>
       <c r="K58" s="2"/>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A59" s="17"/>
-      <c r="B59" s="16"/>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A59" s="26"/>
+      <c r="B59" s="32"/>
       <c r="C59" s="2">
         <v>57</v>
       </c>
@@ -2840,19 +2840,19 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J59" s="2">
         <v>2</v>
       </c>
       <c r="K59" s="2"/>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A60" s="17"/>
-      <c r="B60" s="16"/>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A60" s="26"/>
+      <c r="B60" s="32"/>
       <c r="C60" s="2">
         <v>58</v>
       </c>
@@ -2870,19 +2870,19 @@
         <v>9.7222222222221877E-3</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J60" s="2">
         <v>3</v>
       </c>
       <c r="K60" s="2"/>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A61" s="17"/>
-      <c r="B61" s="16"/>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A61" s="26"/>
+      <c r="B61" s="32"/>
       <c r="C61" s="2">
         <v>59</v>
       </c>
@@ -2900,19 +2900,19 @@
         <v>9.7222222222222987E-3</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="J61" s="2">
         <v>2</v>
       </c>
       <c r="K61" s="2"/>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A62" s="17"/>
-      <c r="B62" s="16"/>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A62" s="26"/>
+      <c r="B62" s="32"/>
       <c r="C62" s="2">
         <v>60</v>
       </c>
@@ -2930,337 +2930,342 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="J62" s="2">
         <v>3</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A63" s="17" t="s">
-        <v>150</v>
-      </c>
-      <c r="B63" s="24">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A63" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="B63" s="33">
         <v>45807</v>
       </c>
-      <c r="C63" s="25">
+      <c r="C63" s="14">
         <v>61</v>
       </c>
-      <c r="D63" s="25">
+      <c r="D63" s="14">
         <v>4321</v>
       </c>
-      <c r="E63" s="26">
+      <c r="E63" s="15">
         <v>0.70902777777777781</v>
       </c>
-      <c r="F63" s="26">
+      <c r="F63" s="15">
         <v>0.71944444444444444</v>
       </c>
-      <c r="G63" s="26">
+      <c r="G63" s="15">
         <f t="shared" si="0"/>
         <v>1.041666666666663E-2</v>
       </c>
-      <c r="H63" s="25" t="s">
+      <c r="H63" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="I63" s="14"/>
+      <c r="J63" s="14"/>
+      <c r="K63" s="14" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A64" s="26"/>
+      <c r="B64" s="34"/>
+      <c r="C64" s="14">
+        <v>62</v>
+      </c>
+      <c r="D64" s="14">
+        <v>1298</v>
+      </c>
+      <c r="E64" s="15">
+        <v>0.6</v>
+      </c>
+      <c r="F64" s="15">
+        <v>0.61041666666666672</v>
+      </c>
+      <c r="G64" s="15">
+        <f t="shared" si="0"/>
+        <v>1.0416666666666741E-2</v>
+      </c>
+      <c r="H64" s="14"/>
+      <c r="I64" s="14"/>
+      <c r="J64" s="14"/>
+      <c r="K64" s="14" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A65" s="26"/>
+      <c r="B65" s="34"/>
+      <c r="C65" s="14">
+        <v>63</v>
+      </c>
+      <c r="D65" s="14">
+        <v>34.1</v>
+      </c>
+      <c r="E65" s="15">
+        <v>0.61875000000000002</v>
+      </c>
+      <c r="F65" s="15">
+        <v>0.62916666666666665</v>
+      </c>
+      <c r="G65" s="15">
+        <f t="shared" si="0"/>
+        <v>1.041666666666663E-2</v>
+      </c>
+      <c r="H65" s="14"/>
+      <c r="I65" s="14"/>
+      <c r="J65" s="14"/>
+      <c r="K65" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="I63" s="25"/>
-      <c r="J63" s="25"/>
-      <c r="K63" s="25" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A64" s="17"/>
-      <c r="B64" s="27"/>
-      <c r="C64" s="25">
-        <v>62</v>
-      </c>
-      <c r="D64" s="25">
-        <v>1298</v>
-      </c>
-      <c r="E64" s="26">
-        <v>0.6</v>
-      </c>
-      <c r="F64" s="26">
-        <v>0.61041666666666672</v>
-      </c>
-      <c r="G64" s="26">
-        <f t="shared" si="0"/>
-        <v>1.0416666666666741E-2</v>
-      </c>
-      <c r="H64" s="25"/>
-      <c r="I64" s="25"/>
-      <c r="J64" s="25"/>
-      <c r="K64" s="25" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A65" s="17"/>
-      <c r="B65" s="27"/>
-      <c r="C65" s="25">
-        <v>63</v>
-      </c>
-      <c r="D65" s="25">
-        <v>34.1</v>
-      </c>
-      <c r="E65" s="26">
-        <v>0.61875000000000002</v>
-      </c>
-      <c r="F65" s="26">
-        <v>0.62916666666666665</v>
-      </c>
-      <c r="G65" s="26">
-        <f t="shared" si="0"/>
-        <v>1.041666666666663E-2</v>
-      </c>
-      <c r="H65" s="25"/>
-      <c r="I65" s="25"/>
-      <c r="J65" s="25"/>
-      <c r="K65" s="25" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A66" s="17"/>
-      <c r="B66" s="28"/>
-      <c r="C66" s="25">
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A66" s="26"/>
+      <c r="B66" s="35"/>
+      <c r="C66" s="14">
         <v>64</v>
       </c>
-      <c r="D66" s="25">
+      <c r="D66" s="14">
         <v>197.8</v>
       </c>
-      <c r="E66" s="26">
+      <c r="E66" s="15">
         <v>0.70138888888888884</v>
       </c>
-      <c r="F66" s="26">
+      <c r="F66" s="15">
         <v>0.71180555555555558</v>
       </c>
-      <c r="G66" s="26">
+      <c r="G66" s="15">
         <f>F66-E66</f>
         <v>1.0416666666666741E-2</v>
       </c>
-      <c r="H66" s="25" t="s">
-        <v>143</v>
-      </c>
-      <c r="I66" s="25"/>
-      <c r="J66" s="25"/>
-      <c r="K66" s="25"/>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A67" s="17" t="s">
+      <c r="H66" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="I66" s="14"/>
+      <c r="J66" s="14"/>
+      <c r="K66" s="14"/>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A67" s="26" t="s">
+        <v>147</v>
+      </c>
+      <c r="B67" s="36">
+        <v>46173</v>
+      </c>
+      <c r="C67" s="16">
+        <v>65</v>
+      </c>
+      <c r="D67" s="16"/>
+      <c r="E67" s="16"/>
+      <c r="F67" s="16"/>
+      <c r="G67" s="16"/>
+      <c r="H67" s="16"/>
+      <c r="I67" s="16"/>
+      <c r="J67" s="16"/>
+      <c r="K67" s="16"/>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A68" s="26"/>
+      <c r="B68" s="37"/>
+      <c r="C68" s="16">
+        <v>66</v>
+      </c>
+      <c r="D68" s="16"/>
+      <c r="E68" s="16"/>
+      <c r="F68" s="16"/>
+      <c r="G68" s="16"/>
+      <c r="H68" s="16"/>
+      <c r="I68" s="16"/>
+      <c r="J68" s="16"/>
+      <c r="K68" s="16"/>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A69" s="26"/>
+      <c r="B69" s="37"/>
+      <c r="C69" s="16">
+        <v>67</v>
+      </c>
+      <c r="D69" s="16"/>
+      <c r="E69" s="16"/>
+      <c r="F69" s="16"/>
+      <c r="G69" s="16"/>
+      <c r="H69" s="16"/>
+      <c r="I69" s="16"/>
+      <c r="J69" s="16"/>
+      <c r="K69" s="16"/>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A70" s="26"/>
+      <c r="B70" s="38"/>
+      <c r="C70" s="16">
+        <v>68</v>
+      </c>
+      <c r="D70" s="16"/>
+      <c r="E70" s="16"/>
+      <c r="F70" s="16"/>
+      <c r="G70" s="16"/>
+      <c r="H70" s="16"/>
+      <c r="I70" s="16"/>
+      <c r="J70" s="16"/>
+      <c r="K70" s="16"/>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A71" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="B67" s="29">
-        <v>46173</v>
-      </c>
-      <c r="C67" s="30">
-        <v>65</v>
-      </c>
-      <c r="D67" s="30"/>
-      <c r="E67" s="30"/>
-      <c r="F67" s="30"/>
-      <c r="G67" s="30"/>
-      <c r="H67" s="30"/>
-      <c r="I67" s="30"/>
-      <c r="J67" s="30"/>
-      <c r="K67" s="30"/>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A68" s="17"/>
-      <c r="B68" s="31"/>
-      <c r="C68" s="30">
-        <v>66</v>
-      </c>
-      <c r="D68" s="30"/>
-      <c r="E68" s="30"/>
-      <c r="F68" s="30"/>
-      <c r="G68" s="30"/>
-      <c r="H68" s="30"/>
-      <c r="I68" s="30"/>
-      <c r="J68" s="30"/>
-      <c r="K68" s="30"/>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A69" s="17"/>
-      <c r="B69" s="31"/>
-      <c r="C69" s="30">
-        <v>67</v>
-      </c>
-      <c r="D69" s="30"/>
-      <c r="E69" s="30"/>
-      <c r="F69" s="30"/>
-      <c r="G69" s="30"/>
-      <c r="H69" s="30"/>
-      <c r="I69" s="30"/>
-      <c r="J69" s="30"/>
-      <c r="K69" s="30"/>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A70" s="17"/>
-      <c r="B70" s="32"/>
-      <c r="C70" s="30">
-        <v>68</v>
-      </c>
-      <c r="D70" s="30"/>
-      <c r="E70" s="30"/>
-      <c r="F70" s="30"/>
-      <c r="G70" s="30"/>
-      <c r="H70" s="30"/>
-      <c r="I70" s="30"/>
-      <c r="J70" s="30"/>
-      <c r="K70" s="30"/>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A71" s="21" t="s">
-        <v>151</v>
-      </c>
-      <c r="B71" s="33">
+      <c r="B71" s="19">
         <v>46174</v>
       </c>
-      <c r="C71" s="34">
+      <c r="C71" s="17">
         <v>69</v>
       </c>
-      <c r="D71" s="34"/>
-      <c r="E71" s="34"/>
-      <c r="F71" s="34"/>
-      <c r="G71" s="34"/>
-      <c r="H71" s="34"/>
-      <c r="I71" s="34"/>
-      <c r="J71" s="34"/>
-      <c r="K71" s="34"/>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A72" s="22"/>
-      <c r="B72" s="35"/>
-      <c r="C72" s="34">
+      <c r="D71" s="17"/>
+      <c r="E71" s="17"/>
+      <c r="F71" s="17"/>
+      <c r="G71" s="17"/>
+      <c r="H71" s="17"/>
+      <c r="I71" s="17"/>
+      <c r="J71" s="17"/>
+      <c r="K71" s="17"/>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A72" s="24"/>
+      <c r="B72" s="20"/>
+      <c r="C72" s="17">
         <v>70</v>
       </c>
-      <c r="D72" s="34"/>
-      <c r="E72" s="34"/>
-      <c r="F72" s="34"/>
-      <c r="G72" s="34"/>
-      <c r="H72" s="34"/>
-      <c r="I72" s="34"/>
-      <c r="J72" s="34"/>
-      <c r="K72" s="34"/>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A73" s="22"/>
-      <c r="B73" s="35"/>
-      <c r="C73" s="34">
+      <c r="D72" s="17"/>
+      <c r="E72" s="17"/>
+      <c r="F72" s="17"/>
+      <c r="G72" s="17"/>
+      <c r="H72" s="17"/>
+      <c r="I72" s="17"/>
+      <c r="J72" s="17"/>
+      <c r="K72" s="17"/>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A73" s="24"/>
+      <c r="B73" s="20"/>
+      <c r="C73" s="17">
         <v>71</v>
       </c>
-      <c r="D73" s="34"/>
-      <c r="E73" s="34"/>
-      <c r="F73" s="34"/>
-      <c r="G73" s="34"/>
-      <c r="H73" s="34"/>
-      <c r="I73" s="34"/>
-      <c r="J73" s="34"/>
-      <c r="K73" s="34"/>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A74" s="22"/>
-      <c r="B74" s="35"/>
-      <c r="C74" s="34">
+      <c r="D73" s="17"/>
+      <c r="E73" s="17"/>
+      <c r="F73" s="17"/>
+      <c r="G73" s="17"/>
+      <c r="H73" s="17"/>
+      <c r="I73" s="17"/>
+      <c r="J73" s="17"/>
+      <c r="K73" s="17"/>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A74" s="24"/>
+      <c r="B74" s="20"/>
+      <c r="C74" s="17">
         <v>72</v>
       </c>
-      <c r="D74" s="34"/>
-      <c r="E74" s="34"/>
-      <c r="F74" s="34"/>
-      <c r="G74" s="34"/>
-      <c r="H74" s="34"/>
-      <c r="I74" s="34"/>
-      <c r="J74" s="34"/>
-      <c r="K74" s="34"/>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A75" s="22"/>
-      <c r="B75" s="35"/>
-      <c r="C75" s="34">
+      <c r="D74" s="17"/>
+      <c r="E74" s="17"/>
+      <c r="F74" s="17"/>
+      <c r="G74" s="17"/>
+      <c r="H74" s="17"/>
+      <c r="I74" s="17"/>
+      <c r="J74" s="17"/>
+      <c r="K74" s="17"/>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A75" s="24"/>
+      <c r="B75" s="20"/>
+      <c r="C75" s="17">
         <v>73</v>
       </c>
-      <c r="D75" s="34"/>
-      <c r="E75" s="34"/>
-      <c r="F75" s="34"/>
-      <c r="G75" s="34"/>
-      <c r="H75" s="34"/>
-      <c r="I75" s="34"/>
-      <c r="J75" s="34"/>
-      <c r="K75" s="34"/>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A76" s="23"/>
-      <c r="B76" s="36"/>
-      <c r="C76" s="34">
+      <c r="D75" s="17"/>
+      <c r="E75" s="17"/>
+      <c r="F75" s="17"/>
+      <c r="G75" s="17"/>
+      <c r="H75" s="17"/>
+      <c r="I75" s="17"/>
+      <c r="J75" s="17"/>
+      <c r="K75" s="17"/>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A76" s="25"/>
+      <c r="B76" s="21"/>
+      <c r="C76" s="17">
         <v>74</v>
       </c>
-      <c r="D76" s="34"/>
-      <c r="E76" s="34"/>
-      <c r="F76" s="34"/>
-      <c r="G76" s="34"/>
-      <c r="H76" s="34"/>
-      <c r="I76" s="34"/>
-      <c r="J76" s="34"/>
-      <c r="K76" s="34"/>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A77" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B77" s="37">
+      <c r="D76" s="17"/>
+      <c r="E76" s="17"/>
+      <c r="F76" s="17"/>
+      <c r="G76" s="17"/>
+      <c r="H76" s="17"/>
+      <c r="I76" s="17"/>
+      <c r="J76" s="17"/>
+      <c r="K76" s="17"/>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A77" s="26" t="s">
+        <v>150</v>
+      </c>
+      <c r="B77" s="22">
         <v>46176</v>
       </c>
-      <c r="C77" s="38">
+      <c r="C77" s="18">
         <v>75</v>
       </c>
-      <c r="D77" s="38"/>
-      <c r="E77" s="38"/>
-      <c r="F77" s="38"/>
-      <c r="G77" s="38"/>
-      <c r="H77" s="38"/>
-      <c r="I77" s="38"/>
-      <c r="J77" s="38"/>
-      <c r="K77" s="38"/>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A78" s="17"/>
-      <c r="B78" s="37"/>
-      <c r="C78" s="38">
+      <c r="D77" s="18"/>
+      <c r="E77" s="18"/>
+      <c r="F77" s="18"/>
+      <c r="G77" s="18"/>
+      <c r="H77" s="18"/>
+      <c r="I77" s="18"/>
+      <c r="J77" s="18"/>
+      <c r="K77" s="18"/>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A78" s="26"/>
+      <c r="B78" s="22"/>
+      <c r="C78" s="18">
         <v>76</v>
       </c>
-      <c r="D78" s="38"/>
-      <c r="E78" s="38"/>
-      <c r="F78" s="38"/>
-      <c r="G78" s="38"/>
-      <c r="H78" s="38"/>
-      <c r="I78" s="38"/>
-      <c r="J78" s="38"/>
-      <c r="K78" s="38"/>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A79" s="17"/>
-      <c r="B79" s="37"/>
-      <c r="C79" s="38">
+      <c r="D78" s="18"/>
+      <c r="E78" s="18"/>
+      <c r="F78" s="18"/>
+      <c r="G78" s="18"/>
+      <c r="H78" s="18"/>
+      <c r="I78" s="18"/>
+      <c r="J78" s="18"/>
+      <c r="K78" s="18"/>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A79" s="26"/>
+      <c r="B79" s="22"/>
+      <c r="C79" s="18">
         <v>77</v>
       </c>
-      <c r="D79" s="38"/>
-      <c r="E79" s="38"/>
-      <c r="F79" s="38"/>
-      <c r="G79" s="38"/>
-      <c r="H79" s="38"/>
-      <c r="I79" s="38"/>
-      <c r="J79" s="38"/>
-      <c r="K79" s="38"/>
+      <c r="D79" s="18"/>
+      <c r="E79" s="18"/>
+      <c r="F79" s="18"/>
+      <c r="G79" s="18"/>
+      <c r="H79" s="18"/>
+      <c r="I79" s="18"/>
+      <c r="J79" s="18"/>
+      <c r="K79" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="B43:B46"/>
+    <mergeCell ref="B47:B52"/>
+    <mergeCell ref="B53:B62"/>
+    <mergeCell ref="B63:B66"/>
+    <mergeCell ref="B67:B70"/>
     <mergeCell ref="B71:B76"/>
     <mergeCell ref="B77:B79"/>
     <mergeCell ref="A71:A76"/>
@@ -3277,11 +3282,6 @@
     <mergeCell ref="A53:A62"/>
     <mergeCell ref="A63:A66"/>
     <mergeCell ref="A67:A70"/>
-    <mergeCell ref="B43:B46"/>
-    <mergeCell ref="B47:B52"/>
-    <mergeCell ref="B53:B62"/>
-    <mergeCell ref="B63:B66"/>
-    <mergeCell ref="B67:B70"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3292,13 +3292,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39518290-7C76-4FD3-8499-94D8E27AC7FD}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="3" width="13.44140625" customWidth="1"/>
+    <col min="2" max="3" width="13.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>50</v>
       </c>
@@ -3309,7 +3309,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -3320,7 +3320,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>3</v>
       </c>
@@ -3331,7 +3331,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>5</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>7</v>
       </c>
@@ -3353,7 +3353,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>9</v>
       </c>
@@ -3364,7 +3364,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>11</v>
       </c>
@@ -3375,7 +3375,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>13</v>
       </c>
@@ -3386,7 +3386,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>15</v>
       </c>
@@ -3397,7 +3397,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>17</v>
       </c>
@@ -3408,7 +3408,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>19</v>
       </c>

</xml_diff>

<commit_message>
Update density boxplot labels for Branchlet and Combined Bark plots
- Rename 'Stringybark Total' to 'Combined Stringybark' and 'Total' to 'Combined all bark' in density_combined_bark.py
- Fix path to Candlebark dataset in density_combined_bark.py to correctly include it in the plot
- Rename 'Total' category to 'Combined all' in Branchlet density boxplot.py
- Regenerate both boxplot figures
</commit_message>
<xml_diff>
--- a/Branchlet/experiment note.xlsx
+++ b/Branchlet/experiment note.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud-my.sharepoint.com/personal/haninhn_student_unimelb_edu_au/Documents/Documents/Chapter 2/Chapter 2 data/Branchlet/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud-my.sharepoint.com/personal/haninhn_student_unimelb_edu_au/Documents/Documents/Chapter 2/Chapter 2 data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{75BA6992-2943-534C-A194-6274ADBAC4E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D5DF9DC-24D4-E14D-8CF7-615D18A29C85}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{AAFCE635-D9F3-D24B-A1CF-31A5BDD9C714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C526FA9-83D1-0442-BB01-8ECA4944652D}"/>
   <bookViews>
-    <workbookView xWindow="5920" yWindow="-18900" windowWidth="22280" windowHeight="14620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34860" yWindow="-4820" windowWidth="29420" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -252,12 +252,6 @@
     <t>0424_10</t>
   </si>
   <si>
-    <t>Twigs (1)</t>
-  </si>
-  <si>
-    <t>Twigs (2)</t>
-  </si>
-  <si>
     <t>Pine</t>
   </si>
   <si>
@@ -496,6 +490,12 @@
   </si>
   <si>
     <t>0505_01</t>
+  </si>
+  <si>
+    <t>Additional test</t>
+  </si>
+  <si>
+    <t>Twigs</t>
   </si>
 </sst>
 </file>
@@ -684,6 +684,33 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="16" fontId="0" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -715,33 +742,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1047,13 +1047,13 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B2" s="13" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D2" s="13" t="s">
         <v>1</v>
@@ -1081,10 +1081,10 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="26" t="s">
-        <v>144</v>
-      </c>
-      <c r="B3" s="27">
+      <c r="A3" s="35" t="s">
+        <v>142</v>
+      </c>
+      <c r="B3" s="36">
         <v>45743</v>
       </c>
       <c r="C3" s="2">
@@ -1115,7 +1115,7 @@
       <c r="K3" s="2"/>
       <c r="L3">
         <f>J3+J5+J7+J9+J11+J13+J15+J17+J19+J21</f>
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="M3">
         <f>J4+J6+J8+J10+J12+J14+J16+J18+J20+J22</f>
@@ -1123,8 +1123,8 @@
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="26"/>
-      <c r="B4" s="27"/>
+      <c r="A4" s="35"/>
+      <c r="B4" s="36"/>
       <c r="C4" s="4">
         <v>2</v>
       </c>
@@ -1153,8 +1153,8 @@
       <c r="K4" s="4"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="26"/>
-      <c r="B5" s="27"/>
+      <c r="A5" s="35"/>
+      <c r="B5" s="36"/>
       <c r="C5" s="2">
         <v>3</v>
       </c>
@@ -1178,13 +1178,13 @@
         <v>15</v>
       </c>
       <c r="J5" s="2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K5" s="2"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="26"/>
-      <c r="B6" s="27"/>
+      <c r="A6" s="35"/>
+      <c r="B6" s="36"/>
       <c r="C6" s="4">
         <v>4</v>
       </c>
@@ -1213,8 +1213,8 @@
       <c r="K6" s="4"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="26"/>
-      <c r="B7" s="27"/>
+      <c r="A7" s="35"/>
+      <c r="B7" s="36"/>
       <c r="C7" s="2">
         <v>5</v>
       </c>
@@ -1243,8 +1243,8 @@
       <c r="K7" s="2"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="26"/>
-      <c r="B8" s="27"/>
+      <c r="A8" s="35"/>
+      <c r="B8" s="36"/>
       <c r="C8" s="4">
         <v>6</v>
       </c>
@@ -1265,7 +1265,7 @@
         <v>19</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J8" s="4">
         <v>6</v>
@@ -1273,8 +1273,8 @@
       <c r="K8" s="4"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="26"/>
-      <c r="B9" s="27"/>
+      <c r="A9" s="35"/>
+      <c r="B9" s="36"/>
       <c r="C9" s="2">
         <v>7</v>
       </c>
@@ -1303,8 +1303,8 @@
       <c r="K9" s="2"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" s="26"/>
-      <c r="B10" s="27"/>
+      <c r="A10" s="35"/>
+      <c r="B10" s="36"/>
       <c r="C10" s="4">
         <v>8</v>
       </c>
@@ -1333,8 +1333,8 @@
       <c r="K10" s="4"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A11" s="26"/>
-      <c r="B11" s="27">
+      <c r="A11" s="35"/>
+      <c r="B11" s="36">
         <v>45748</v>
       </c>
       <c r="C11" s="2">
@@ -1365,8 +1365,8 @@
       <c r="K11" s="2"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A12" s="26"/>
-      <c r="B12" s="27"/>
+      <c r="A12" s="35"/>
+      <c r="B12" s="36"/>
       <c r="C12" s="4">
         <v>10</v>
       </c>
@@ -1395,8 +1395,8 @@
       <c r="K12" s="4"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A13" s="26"/>
-      <c r="B13" s="27"/>
+      <c r="A13" s="35"/>
+      <c r="B13" s="36"/>
       <c r="C13" s="2">
         <v>11</v>
       </c>
@@ -1425,8 +1425,8 @@
       <c r="K13" s="2"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="26"/>
-      <c r="B14" s="27"/>
+      <c r="A14" s="35"/>
+      <c r="B14" s="36"/>
       <c r="C14" s="4">
         <v>12</v>
       </c>
@@ -1455,8 +1455,8 @@
       <c r="K14" s="4"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A15" s="26"/>
-      <c r="B15" s="27"/>
+      <c r="A15" s="35"/>
+      <c r="B15" s="36"/>
       <c r="C15" s="2">
         <v>13</v>
       </c>
@@ -1485,8 +1485,8 @@
       <c r="K15" s="2"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="26"/>
-      <c r="B16" s="27"/>
+      <c r="A16" s="35"/>
+      <c r="B16" s="36"/>
       <c r="C16" s="4">
         <v>14</v>
       </c>
@@ -1515,8 +1515,8 @@
       <c r="K16" s="4"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A17" s="26"/>
-      <c r="B17" s="27"/>
+      <c r="A17" s="35"/>
+      <c r="B17" s="36"/>
       <c r="C17" s="2">
         <v>15</v>
       </c>
@@ -1545,8 +1545,8 @@
       <c r="K17" s="2"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A18" s="26"/>
-      <c r="B18" s="27"/>
+      <c r="A18" s="35"/>
+      <c r="B18" s="36"/>
       <c r="C18" s="4">
         <v>16</v>
       </c>
@@ -1575,8 +1575,8 @@
       <c r="K18" s="4"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" s="26"/>
-      <c r="B19" s="27"/>
+      <c r="A19" s="35"/>
+      <c r="B19" s="36"/>
       <c r="C19" s="2">
         <v>17</v>
       </c>
@@ -1605,8 +1605,8 @@
       <c r="K19" s="2"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A20" s="26"/>
-      <c r="B20" s="27"/>
+      <c r="A20" s="35"/>
+      <c r="B20" s="36"/>
       <c r="C20" s="4">
         <v>18</v>
       </c>
@@ -1635,8 +1635,8 @@
       <c r="K20" s="4"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A21" s="26"/>
-      <c r="B21" s="27"/>
+      <c r="A21" s="35"/>
+      <c r="B21" s="36"/>
       <c r="C21" s="2">
         <v>19</v>
       </c>
@@ -1667,8 +1667,8 @@
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A22" s="26"/>
-      <c r="B22" s="27"/>
+      <c r="A22" s="35"/>
+      <c r="B22" s="36"/>
       <c r="C22" s="4">
         <v>20</v>
       </c>
@@ -1697,10 +1697,10 @@
       <c r="K22" s="4"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A23" s="26" t="s">
-        <v>71</v>
-      </c>
-      <c r="B23" s="28">
+      <c r="A23" s="35" t="s">
+        <v>151</v>
+      </c>
+      <c r="B23" s="37">
         <v>45763</v>
       </c>
       <c r="C23" s="7">
@@ -1720,7 +1720,7 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="I23" s="7" t="s">
         <v>61</v>
@@ -1737,8 +1737,8 @@
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A24" s="26"/>
-      <c r="B24" s="28"/>
+      <c r="A24" s="35"/>
+      <c r="B24" s="37"/>
       <c r="C24" s="7">
         <v>22</v>
       </c>
@@ -1767,8 +1767,8 @@
       <c r="K24" s="7"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A25" s="26"/>
-      <c r="B25" s="28"/>
+      <c r="A25" s="35"/>
+      <c r="B25" s="37"/>
       <c r="C25" s="7">
         <v>23</v>
       </c>
@@ -1797,8 +1797,8 @@
       <c r="K25" s="7"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A26" s="26"/>
-      <c r="B26" s="28"/>
+      <c r="A26" s="35"/>
+      <c r="B26" s="37"/>
       <c r="C26" s="7">
         <v>24</v>
       </c>
@@ -1827,8 +1827,8 @@
       <c r="K26" s="7"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A27" s="26"/>
-      <c r="B27" s="28"/>
+      <c r="A27" s="35"/>
+      <c r="B27" s="37"/>
       <c r="C27" s="7">
         <v>25</v>
       </c>
@@ -1857,8 +1857,8 @@
       <c r="K27" s="7"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A28" s="26"/>
-      <c r="B28" s="28"/>
+      <c r="A28" s="35"/>
+      <c r="B28" s="37"/>
       <c r="C28" s="7">
         <v>26</v>
       </c>
@@ -1887,8 +1887,8 @@
       <c r="K28" s="7"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A29" s="26"/>
-      <c r="B29" s="28"/>
+      <c r="A29" s="35"/>
+      <c r="B29" s="37"/>
       <c r="C29" s="7">
         <v>27</v>
       </c>
@@ -1917,8 +1917,8 @@
       <c r="K29" s="7"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A30" s="26"/>
-      <c r="B30" s="28"/>
+      <c r="A30" s="35"/>
+      <c r="B30" s="37"/>
       <c r="C30" s="7">
         <v>28</v>
       </c>
@@ -1947,8 +1947,8 @@
       <c r="K30" s="7"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A31" s="26"/>
-      <c r="B31" s="28"/>
+      <c r="A31" s="35"/>
+      <c r="B31" s="37"/>
       <c r="C31" s="7">
         <v>29</v>
       </c>
@@ -1977,8 +1977,8 @@
       <c r="K31" s="7"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A32" s="26"/>
-      <c r="B32" s="28"/>
+      <c r="A32" s="35"/>
+      <c r="B32" s="37"/>
       <c r="C32" s="7">
         <v>30</v>
       </c>
@@ -2007,10 +2007,10 @@
       <c r="K32" s="7"/>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A33" s="26" t="s">
-        <v>72</v>
-      </c>
-      <c r="B33" s="29">
+      <c r="A33" s="35" t="s">
+        <v>152</v>
+      </c>
+      <c r="B33" s="38">
         <v>45778</v>
       </c>
       <c r="C33" s="9">
@@ -2030,23 +2030,23 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I33" s="9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="J33" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K33" s="9"/>
       <c r="L33">
         <f>SUM(J33:J42)</f>
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A34" s="26"/>
-      <c r="B34" s="29"/>
+      <c r="A34" s="35"/>
+      <c r="B34" s="38"/>
       <c r="C34" s="9">
         <v>32</v>
       </c>
@@ -2064,10 +2064,10 @@
         <v>1.0416666666666741E-2</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="I34" s="9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="J34" s="9">
         <v>4</v>
@@ -2075,8 +2075,8 @@
       <c r="K34" s="9"/>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A35" s="26"/>
-      <c r="B35" s="29"/>
+      <c r="A35" s="35"/>
+      <c r="B35" s="38"/>
       <c r="C35" s="9">
         <v>33</v>
       </c>
@@ -2094,21 +2094,21 @@
         <v>1.0416666666666741E-2</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="I35" s="9" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J35" s="9">
         <v>3</v>
       </c>
       <c r="K35" s="9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A36" s="26"/>
-      <c r="B36" s="29"/>
+      <c r="A36" s="35"/>
+      <c r="B36" s="38"/>
       <c r="C36" s="9">
         <v>34</v>
       </c>
@@ -2126,10 +2126,10 @@
         <v>1.0416666666666741E-2</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I36" s="9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J36" s="9">
         <v>3</v>
@@ -2137,8 +2137,8 @@
       <c r="K36" s="9"/>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A37" s="26"/>
-      <c r="B37" s="29"/>
+      <c r="A37" s="35"/>
+      <c r="B37" s="38"/>
       <c r="C37" s="9">
         <v>35</v>
       </c>
@@ -2156,10 +2156,10 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H37" s="9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I37" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="J37" s="9">
         <v>3</v>
@@ -2167,8 +2167,8 @@
       <c r="K37" s="9"/>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A38" s="26"/>
-      <c r="B38" s="29">
+      <c r="A38" s="35"/>
+      <c r="B38" s="38">
         <v>45779</v>
       </c>
       <c r="C38" s="9">
@@ -2188,21 +2188,21 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I38" s="9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="J38" s="9">
         <v>2</v>
       </c>
       <c r="K38" s="9" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A39" s="26"/>
-      <c r="B39" s="29"/>
+      <c r="A39" s="35"/>
+      <c r="B39" s="38"/>
       <c r="C39" s="9">
         <v>37</v>
       </c>
@@ -2220,10 +2220,10 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I39" s="9" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="J39" s="9">
         <v>3</v>
@@ -2231,8 +2231,8 @@
       <c r="K39" s="9"/>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A40" s="26"/>
-      <c r="B40" s="29"/>
+      <c r="A40" s="35"/>
+      <c r="B40" s="38"/>
       <c r="C40" s="9">
         <v>38</v>
       </c>
@@ -2250,10 +2250,10 @@
         <v>1.0416666666666741E-2</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="I40" s="9" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="J40" s="9">
         <v>2</v>
@@ -2261,8 +2261,8 @@
       <c r="K40" s="9"/>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A41" s="26"/>
-      <c r="B41" s="29"/>
+      <c r="A41" s="35"/>
+      <c r="B41" s="38"/>
       <c r="C41" s="9">
         <v>39</v>
       </c>
@@ -2280,10 +2280,10 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H41" s="9" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="I41" s="9" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J41" s="9">
         <v>3</v>
@@ -2291,8 +2291,8 @@
       <c r="K41" s="9"/>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A42" s="26"/>
-      <c r="B42" s="29"/>
+      <c r="A42" s="35"/>
+      <c r="B42" s="38"/>
       <c r="C42" s="9">
         <v>40</v>
       </c>
@@ -2310,23 +2310,23 @@
         <v>8.3333333333333037E-3</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I42" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="J42" s="9">
         <v>3</v>
       </c>
       <c r="K42" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A43" s="26" t="s">
-        <v>73</v>
-      </c>
-      <c r="B43" s="30">
+      <c r="A43" s="35" t="s">
+        <v>71</v>
+      </c>
+      <c r="B43" s="19">
         <v>45792</v>
       </c>
       <c r="C43" s="10">
@@ -2346,10 +2346,10 @@
         <v>9.0277777777777457E-3</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="I43" s="10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="J43" s="10">
         <v>2</v>
@@ -2361,8 +2361,8 @@
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A44" s="26"/>
-      <c r="B44" s="31"/>
+      <c r="A44" s="35"/>
+      <c r="B44" s="20"/>
       <c r="C44" s="10">
         <v>42</v>
       </c>
@@ -2380,10 +2380,10 @@
         <v>1.0416666666666741E-2</v>
       </c>
       <c r="H44" s="10" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="J44" s="10">
         <v>2</v>
@@ -2391,8 +2391,8 @@
       <c r="K44" s="10"/>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A45" s="26"/>
-      <c r="B45" s="31"/>
+      <c r="A45" s="35"/>
+      <c r="B45" s="20"/>
       <c r="C45" s="10">
         <v>43</v>
       </c>
@@ -2410,10 +2410,10 @@
         <v>8.3333333333333037E-3</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I45" s="10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J45" s="10">
         <v>3</v>
@@ -2421,8 +2421,8 @@
       <c r="K45" s="10"/>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A46" s="26"/>
-      <c r="B46" s="31"/>
+      <c r="A46" s="35"/>
+      <c r="B46" s="20"/>
       <c r="C46" s="10">
         <v>44</v>
       </c>
@@ -2440,10 +2440,10 @@
         <v>9.0277777777777457E-3</v>
       </c>
       <c r="H46" s="10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J46" s="10">
         <v>2</v>
@@ -2451,8 +2451,8 @@
       <c r="K46" s="10"/>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A47" s="26"/>
-      <c r="B47" s="30">
+      <c r="A47" s="35"/>
+      <c r="B47" s="19">
         <v>45793</v>
       </c>
       <c r="C47" s="10">
@@ -2472,10 +2472,10 @@
         <v>7.6388888888888618E-3</v>
       </c>
       <c r="H47" s="10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I47" s="10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="J47" s="10">
         <v>2</v>
@@ -2483,8 +2483,8 @@
       <c r="K47" s="10"/>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A48" s="26"/>
-      <c r="B48" s="30"/>
+      <c r="A48" s="35"/>
+      <c r="B48" s="19"/>
       <c r="C48" s="10">
         <v>46</v>
       </c>
@@ -2502,10 +2502,10 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H48" s="10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="J48" s="10">
         <v>2</v>
@@ -2513,8 +2513,8 @@
       <c r="K48" s="10"/>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A49" s="26"/>
-      <c r="B49" s="30"/>
+      <c r="A49" s="35"/>
+      <c r="B49" s="19"/>
       <c r="C49" s="10">
         <v>47</v>
       </c>
@@ -2532,10 +2532,10 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I49" s="10" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J49" s="10">
         <v>3</v>
@@ -2543,8 +2543,8 @@
       <c r="K49" s="10"/>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A50" s="26"/>
-      <c r="B50" s="30"/>
+      <c r="A50" s="35"/>
+      <c r="B50" s="19"/>
       <c r="C50" s="10">
         <v>48</v>
       </c>
@@ -2562,10 +2562,10 @@
         <v>9.7222222222222987E-3</v>
       </c>
       <c r="H50" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="I50" s="10" t="s">
         <v>113</v>
-      </c>
-      <c r="I50" s="10" t="s">
-        <v>115</v>
       </c>
       <c r="J50" s="10">
         <v>2</v>
@@ -2573,8 +2573,8 @@
       <c r="K50" s="10"/>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A51" s="26"/>
-      <c r="B51" s="30"/>
+      <c r="A51" s="35"/>
+      <c r="B51" s="19"/>
       <c r="C51" s="10">
         <v>49</v>
       </c>
@@ -2592,10 +2592,10 @@
         <v>6.9444444444444198E-3</v>
       </c>
       <c r="H51" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I51" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J51" s="10">
         <v>4</v>
@@ -2603,8 +2603,8 @@
       <c r="K51" s="10"/>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A52" s="26"/>
-      <c r="B52" s="30"/>
+      <c r="A52" s="35"/>
+      <c r="B52" s="19"/>
       <c r="C52" s="10">
         <v>50</v>
       </c>
@@ -2622,10 +2622,10 @@
         <v>7.6388888888889728E-3</v>
       </c>
       <c r="H52" s="10" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="J52" s="10">
         <v>3</v>
@@ -2633,10 +2633,10 @@
       <c r="K52" s="10"/>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A53" s="26" t="s">
-        <v>74</v>
-      </c>
-      <c r="B53" s="32">
+      <c r="A53" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="B53" s="21">
         <v>45794</v>
       </c>
       <c r="C53" s="2">
@@ -2656,10 +2656,10 @@
         <v>9.2361111111111116E-2</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J53" s="2">
         <v>2</v>
@@ -2671,8 +2671,8 @@
       </c>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A54" s="26"/>
-      <c r="B54" s="32"/>
+      <c r="A54" s="35"/>
+      <c r="B54" s="21"/>
       <c r="C54" s="2">
         <v>52</v>
       </c>
@@ -2690,10 +2690,10 @@
         <v>1.0416666666666741E-2</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="J54" s="2">
         <v>2</v>
@@ -2701,8 +2701,8 @@
       <c r="K54" s="2"/>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A55" s="26"/>
-      <c r="B55" s="32"/>
+      <c r="A55" s="35"/>
+      <c r="B55" s="21"/>
       <c r="C55" s="2">
         <v>53</v>
       </c>
@@ -2720,10 +2720,10 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J55" s="2">
         <v>2</v>
@@ -2731,8 +2731,8 @@
       <c r="K55" s="2"/>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A56" s="26"/>
-      <c r="B56" s="32"/>
+      <c r="A56" s="35"/>
+      <c r="B56" s="21"/>
       <c r="C56" s="2">
         <v>54</v>
       </c>
@@ -2750,10 +2750,10 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J56" s="2">
         <v>2</v>
@@ -2761,8 +2761,8 @@
       <c r="K56" s="2"/>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A57" s="26"/>
-      <c r="B57" s="32"/>
+      <c r="A57" s="35"/>
+      <c r="B57" s="21"/>
       <c r="C57" s="2">
         <v>55</v>
       </c>
@@ -2780,10 +2780,10 @@
         <v>9.0277777777778567E-3</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J57" s="2">
         <v>3</v>
@@ -2791,8 +2791,8 @@
       <c r="K57" s="2"/>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A58" s="26"/>
-      <c r="B58" s="32"/>
+      <c r="A58" s="35"/>
+      <c r="B58" s="21"/>
       <c r="C58" s="2">
         <v>56</v>
       </c>
@@ -2810,10 +2810,10 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J58" s="2">
         <v>2</v>
@@ -2821,8 +2821,8 @@
       <c r="K58" s="2"/>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A59" s="26"/>
-      <c r="B59" s="32"/>
+      <c r="A59" s="35"/>
+      <c r="B59" s="21"/>
       <c r="C59" s="2">
         <v>57</v>
       </c>
@@ -2840,10 +2840,10 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="J59" s="2">
         <v>2</v>
@@ -2851,8 +2851,8 @@
       <c r="K59" s="2"/>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A60" s="26"/>
-      <c r="B60" s="32"/>
+      <c r="A60" s="35"/>
+      <c r="B60" s="21"/>
       <c r="C60" s="2">
         <v>58</v>
       </c>
@@ -2870,10 +2870,10 @@
         <v>9.7222222222221877E-3</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J60" s="2">
         <v>3</v>
@@ -2881,8 +2881,8 @@
       <c r="K60" s="2"/>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A61" s="26"/>
-      <c r="B61" s="32"/>
+      <c r="A61" s="35"/>
+      <c r="B61" s="21"/>
       <c r="C61" s="2">
         <v>59</v>
       </c>
@@ -2900,10 +2900,10 @@
         <v>9.7222222222222987E-3</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="J61" s="2">
         <v>2</v>
@@ -2911,8 +2911,8 @@
       <c r="K61" s="2"/>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A62" s="26"/>
-      <c r="B62" s="32"/>
+      <c r="A62" s="35"/>
+      <c r="B62" s="21"/>
       <c r="C62" s="2">
         <v>60</v>
       </c>
@@ -2930,23 +2930,23 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="J62" s="2">
         <v>3</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A63" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="B63" s="33">
+      <c r="A63" s="35" t="s">
+        <v>146</v>
+      </c>
+      <c r="B63" s="22">
         <v>45807</v>
       </c>
       <c r="C63" s="14">
@@ -2966,17 +2966,17 @@
         <v>1.041666666666663E-2</v>
       </c>
       <c r="H63" s="14" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I63" s="14"/>
       <c r="J63" s="14"/>
       <c r="K63" s="14" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A64" s="26"/>
-      <c r="B64" s="34"/>
+      <c r="A64" s="35"/>
+      <c r="B64" s="23"/>
       <c r="C64" s="14">
         <v>62</v>
       </c>
@@ -2997,12 +2997,12 @@
       <c r="I64" s="14"/>
       <c r="J64" s="14"/>
       <c r="K64" s="14" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A65" s="26"/>
-      <c r="B65" s="34"/>
+      <c r="A65" s="35"/>
+      <c r="B65" s="23"/>
       <c r="C65" s="14">
         <v>63</v>
       </c>
@@ -3023,12 +3023,12 @@
       <c r="I65" s="14"/>
       <c r="J65" s="14"/>
       <c r="K65" s="14" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A66" s="26"/>
-      <c r="B66" s="35"/>
+      <c r="A66" s="35"/>
+      <c r="B66" s="24"/>
       <c r="C66" s="14">
         <v>64</v>
       </c>
@@ -3046,17 +3046,17 @@
         <v>1.0416666666666741E-2</v>
       </c>
       <c r="H66" s="14" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="I66" s="14"/>
       <c r="J66" s="14"/>
       <c r="K66" s="14"/>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A67" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="B67" s="36">
+      <c r="A67" s="35" t="s">
+        <v>145</v>
+      </c>
+      <c r="B67" s="25">
         <v>46173</v>
       </c>
       <c r="C67" s="16">
@@ -3072,8 +3072,8 @@
       <c r="K67" s="16"/>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A68" s="26"/>
-      <c r="B68" s="37"/>
+      <c r="A68" s="35"/>
+      <c r="B68" s="26"/>
       <c r="C68" s="16">
         <v>66</v>
       </c>
@@ -3087,8 +3087,8 @@
       <c r="K68" s="16"/>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A69" s="26"/>
-      <c r="B69" s="37"/>
+      <c r="A69" s="35"/>
+      <c r="B69" s="26"/>
       <c r="C69" s="16">
         <v>67</v>
       </c>
@@ -3102,8 +3102,8 @@
       <c r="K69" s="16"/>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A70" s="26"/>
-      <c r="B70" s="38"/>
+      <c r="A70" s="35"/>
+      <c r="B70" s="27"/>
       <c r="C70" s="16">
         <v>68</v>
       </c>
@@ -3117,10 +3117,10 @@
       <c r="K70" s="16"/>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A71" s="23" t="s">
-        <v>149</v>
-      </c>
-      <c r="B71" s="19">
+      <c r="A71" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="B71" s="28">
         <v>46174</v>
       </c>
       <c r="C71" s="17">
@@ -3136,8 +3136,8 @@
       <c r="K71" s="17"/>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A72" s="24"/>
-      <c r="B72" s="20"/>
+      <c r="A72" s="33"/>
+      <c r="B72" s="29"/>
       <c r="C72" s="17">
         <v>70</v>
       </c>
@@ -3151,8 +3151,8 @@
       <c r="K72" s="17"/>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A73" s="24"/>
-      <c r="B73" s="20"/>
+      <c r="A73" s="33"/>
+      <c r="B73" s="29"/>
       <c r="C73" s="17">
         <v>71</v>
       </c>
@@ -3166,8 +3166,8 @@
       <c r="K73" s="17"/>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A74" s="24"/>
-      <c r="B74" s="20"/>
+      <c r="A74" s="33"/>
+      <c r="B74" s="29"/>
       <c r="C74" s="17">
         <v>72</v>
       </c>
@@ -3181,8 +3181,8 @@
       <c r="K74" s="17"/>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A75" s="24"/>
-      <c r="B75" s="20"/>
+      <c r="A75" s="33"/>
+      <c r="B75" s="29"/>
       <c r="C75" s="17">
         <v>73</v>
       </c>
@@ -3196,8 +3196,8 @@
       <c r="K75" s="17"/>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A76" s="25"/>
-      <c r="B76" s="21"/>
+      <c r="A76" s="34"/>
+      <c r="B76" s="30"/>
       <c r="C76" s="17">
         <v>74</v>
       </c>
@@ -3211,10 +3211,10 @@
       <c r="K76" s="17"/>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A77" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="B77" s="22">
+      <c r="A77" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="B77" s="31">
         <v>46176</v>
       </c>
       <c r="C77" s="18">
@@ -3230,8 +3230,8 @@
       <c r="K77" s="18"/>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A78" s="26"/>
-      <c r="B78" s="22"/>
+      <c r="A78" s="35"/>
+      <c r="B78" s="31"/>
       <c r="C78" s="18">
         <v>76</v>
       </c>
@@ -3245,8 +3245,8 @@
       <c r="K78" s="18"/>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A79" s="26"/>
-      <c r="B79" s="22"/>
+      <c r="A79" s="35"/>
+      <c r="B79" s="31"/>
       <c r="C79" s="18">
         <v>77</v>
       </c>
@@ -3261,11 +3261,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B43:B46"/>
-    <mergeCell ref="B47:B52"/>
-    <mergeCell ref="B53:B62"/>
-    <mergeCell ref="B63:B66"/>
-    <mergeCell ref="B67:B70"/>
     <mergeCell ref="B71:B76"/>
     <mergeCell ref="B77:B79"/>
     <mergeCell ref="A71:A76"/>
@@ -3282,6 +3277,11 @@
     <mergeCell ref="A53:A62"/>
     <mergeCell ref="A63:A66"/>
     <mergeCell ref="A67:A70"/>
+    <mergeCell ref="B43:B46"/>
+    <mergeCell ref="B47:B52"/>
+    <mergeCell ref="B53:B62"/>
+    <mergeCell ref="B63:B66"/>
+    <mergeCell ref="B67:B70"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>